<commit_message>
fix(#93): mark Case #006 pnl_pct as N/A (counterfactual sin simulación)
Case 2026-05-27_SPY_counterfactual_006 had pnl_pct =
"PENDING_VALIDATION_TODAY - revisar a las 16:00 ET 27-may" because
the trade was counterfactual (trade_executed='NO'); no real fill
exists in eolo-crop-trades to derive a real PnL from.

Per decision 2026-06-01: mark pnl_pct as "N/A (counterfactual sin
simulación)" definitive and append justification to notes. The value
of this case lives in lesson_learned (qualitative — stop loss requires
multi-confirmation), not in pnl. Black-Scholes simulation rejected to
preserve honesty about counterfactual nature.

Adds one-off script tools/scripts/fix_case_006_pnl_pct.py used to
apply the edit (kept as audit trail; can be removed in follow-up).
Backup written to backups/EOLO_ThetaHarvest_v1.2_pre_case_006_pnl_fix_*.xlsx.

KB validate PASS. list-cases shows 6 cases intact.
</commit_message>
<xml_diff>
--- a/llm_engine_eolo/kb/EOLO_ThetaHarvest_v1.2.xlsx
+++ b/llm_engine_eolo/kb/EOLO_ThetaHarvest_v1.2.xlsx
@@ -3259,7 +3259,7 @@
       </c>
       <c r="BC9" s="49" t="inlineStr">
         <is>
-          <t>CASO EN VIVO - documentado 12:00 ET del 27-may-2026 mientras mercado abierto. Caracteristica unica: incluye PLAN DE GESTION FUTURA explicito (no solo entry). Plan: (1) Entry IC sobre Fibonacci 749/751 secuencial. (2) Recompra parcial 12:00 si no llego a 50-60% profit. (3) STOP LOSS: salida del lado correspondiente si rompe Fibonacci CON triple confirmacion (VIX velocity dispara + volume + RSI cae fuertemente). (4) HOLD: si rompe Fib pero sin confirmacion, aguantar y monitorear. VALIDACION ESPERADA: outcome al cierre 16:00 ET de hoy. [SPRINT #86 cleanup 2026-06-01: case_quality original 'SILVER (LIVE - outcome pending end of day)' normalizado a 'SILVER' para satisfacer enum estricto del validator. Outcome del 27-may pendiente — actualizar pnl_pct con valor real cuando se complete el follow-up.]</t>
+          <t>CASO EN VIVO - documentado 12:00 ET del 27-may-2026 mientras mercado abierto. Caracteristica unica: incluye PLAN DE GESTION FUTURA explicito (no solo entry). Plan: (1) Entry IC sobre Fibonacci 749/751 secuencial. (2) Recompra parcial 12:00 si no llego a 50-60% profit. (3) STOP LOSS: salida del lado correspondiente si rompe Fibonacci CON triple confirmacion (VIX velocity dispara + volume + RSI cae fuertemente). (4) HOLD: si rompe Fib pero sin confirmacion, aguantar y monitorear. VALIDACION ESPERADA: outcome al cierre 16:00 ET de hoy. [SPRINT #86 cleanup 2026-06-01: case_quality original 'SILVER (LIVE - outcome pending end of day)' normalizado a 'SILVER' para satisfacer enum estricto del validator. Outcome del 27-may pendiente — actualizar pnl_pct con valor real cuando se complete el follow-up.] [SPRINT #93 cleanup 2026-06-01: pnl_pct marcado N/A definitivo. Case counterfactual sin trade real (trade_executed=NO); valor cualitativo en lesson_learned. Sin simulación BS para mantener honestidad.]</t>
         </is>
       </c>
       <c r="BD9" s="49" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="BH9" s="49" t="inlineStr">
         <is>
-          <t>PENDING_VALIDATION_TODAY - revisar a las 16:00 ET 27-may</t>
+          <t>N/A (counterfactual sin simulación)</t>
         </is>
       </c>
       <c r="BI9" s="49" t="inlineStr">

</xml_diff>